<commit_message>
fix: move Campo Mourao para mesorregiao Noroeste
- Corrige atribuicao de mesorregiao de Oeste para Noroeste
- Atualiza municipios.geojson, geo_map.json, aggregated.json
- Atualiza municipios_pr.xlsx e mun_PR.json

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/municipios_pr.xlsx
+++ b/data/municipios_pr.xlsx
@@ -5012,7 +5012,7 @@
         <v>735</v>
       </c>
       <c r="E126" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -5216,7 +5216,7 @@
         <v>735</v>
       </c>
       <c r="E138" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="139" spans="1:5">
@@ -6049,7 +6049,7 @@
         <v>735</v>
       </c>
       <c r="E187" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="188" spans="1:5">
@@ -6372,7 +6372,7 @@
         <v>735</v>
       </c>
       <c r="E206" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="207" spans="1:5">
@@ -6389,7 +6389,7 @@
         <v>735</v>
       </c>
       <c r="E207" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -6695,7 +6695,7 @@
         <v>735</v>
       </c>
       <c r="E225" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -6780,7 +6780,7 @@
         <v>735</v>
       </c>
       <c r="E230" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -6882,7 +6882,7 @@
         <v>735</v>
       </c>
       <c r="E236" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="237" spans="1:5">
@@ -6950,7 +6950,7 @@
         <v>735</v>
       </c>
       <c r="E240" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="241" spans="1:5">
@@ -6967,7 +6967,7 @@
         <v>735</v>
       </c>
       <c r="E241" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="242" spans="1:5">
@@ -7086,7 +7086,7 @@
         <v>735</v>
       </c>
       <c r="E248" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="249" spans="1:5">
@@ -7120,7 +7120,7 @@
         <v>735</v>
       </c>
       <c r="E250" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="251" spans="1:5">
@@ -7137,7 +7137,7 @@
         <v>735</v>
       </c>
       <c r="E251" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="252" spans="1:5">
@@ -7239,7 +7239,7 @@
         <v>735</v>
       </c>
       <c r="E257" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="258" spans="1:5">
@@ -7256,7 +7256,7 @@
         <v>735</v>
       </c>
       <c r="E258" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="259" spans="1:5">
@@ -7290,7 +7290,7 @@
         <v>735</v>
       </c>
       <c r="E260" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="261" spans="1:5">
@@ -7307,7 +7307,7 @@
         <v>735</v>
       </c>
       <c r="E261" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="262" spans="1:5">
@@ -7647,7 +7647,7 @@
         <v>735</v>
       </c>
       <c r="E281" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="282" spans="1:5">
@@ -8531,7 +8531,7 @@
         <v>735</v>
       </c>
       <c r="E333" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="334" spans="1:5">
@@ -8633,7 +8633,7 @@
         <v>735</v>
       </c>
       <c r="E339" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="340" spans="1:5">
@@ -8837,7 +8837,7 @@
         <v>735</v>
       </c>
       <c r="E351" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="352" spans="1:5">
@@ -9432,7 +9432,7 @@
         <v>735</v>
       </c>
       <c r="E386" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="387" spans="1:5">
@@ -9449,7 +9449,7 @@
         <v>735</v>
       </c>
       <c r="E387" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="388" spans="1:5">
@@ -9500,7 +9500,7 @@
         <v>735</v>
       </c>
       <c r="E390" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="391" spans="1:5">
@@ -9517,7 +9517,7 @@
         <v>735</v>
       </c>
       <c r="E391" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
     </row>
     <row r="392" spans="1:5">

</xml_diff>